<commit_message>
Retire previous templates and stage new policy PDF catalog
</commit_message>
<xml_diff>
--- a/Base_SASISOPA.xlsx
+++ b/Base_SASISOPA.xlsx
@@ -204,7 +204,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T_Plantillas" displayName="T_Plantillas" ref="A1:C8" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T_Plantillas" displayName="T_Plantillas" ref="A1:C2" headerRowCount="1">
   <autoFilter ref="A1:C8"/>
   <tableColumns count="3">
     <tableColumn id="1" name="plantilla_id"/>
@@ -827,7 +827,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de los siete Word recibidos. No cambies sus identificadores.</t>
+          <t>Nueva base: PROCEDIMIENTO I.pdf, 14 páginas. Las siete plantillas anteriores se retiraron del catálogo activo. El llenado aún está pendiente de adaptar.</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,6 @@
       </c>
       <c r="C2" s="4" t="inlineStr"/>
       <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="C3" s="4" t="n"/>
@@ -4586,7 +4585,6 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>PER-001</t>
@@ -4623,7 +4621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4651,119 +4649,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>POL-I</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7.5-02585 Acuse de Recibo ENE.docx</t>
+          <t>PROCEDIMIENTO I.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Estaciones, Personal, Acuses, Documentos_Entregados, Recepciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>P02</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>7.5- 02585 Plan de Sesion ENE.docx</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Estaciones, Personal, Eventos, Sesiones, Asistentes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>P03</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>10.2-02585 Nota Informativa ENE.docx</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Estaciones, Personal, Eventos, Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>7.1-02585 Difusión Política ENE.docx</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Estaciones, Personal, Eventos, Agenda, Acuerdos, Asistentes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>P05</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>10.2- 02585 Cambios Personal ENE.docx</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Estaciones, Personal, Eventos, Agenda, Acuerdos, Asistentes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1.1.-02585 Revisar Política ENE.docx</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Estaciones, Personal, Eventos, Agenda, Acuerdos, Asistentes</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>P07</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>10.3-02585 Agenda de reunión ENE.docx</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Estaciones, Personal, Eventos, Agenda, Acuerdos, Asistentes</t>
+          <t>Nueva base PDF; llenado pendiente de configurar</t>
         </is>
       </c>
     </row>
@@ -4832,18 +4728,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>P02</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>EVT-001</t>
-        </is>
-      </c>
+          <t>POL-I</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Plan_de_sesion</t>
+          <t>Politica</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -4930,7 +4822,6 @@
           <t>ESTACIÓN DE EJEMPLO</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Sala de juntas</t>
@@ -7024,8 +6915,6 @@
           <t>POR DEFINIR</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" s="4" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
@@ -8656,7 +8545,6 @@
           <t>POR DEFINIR</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>PER-001</t>
@@ -8667,7 +8555,6 @@
           <t>PER-001</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>Borrador</t>
@@ -10891,9 +10778,6 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" s="5" t="n"/>
       <c r="G2" t="inlineStr">
         <is>
@@ -12478,14 +12362,9 @@
           <t>EVT-001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12563,7 +12442,6 @@
       </c>
       <c r="C2" s="4" t="inlineStr"/>
       <c r="D2" s="5" t="n"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>No controlada</t>

</xml_diff>

<commit_message>
Implement native filling of the new fourteen-page policy PDF
</commit_message>
<xml_diff>
--- a/Base_SASISOPA.xlsx
+++ b/Base_SASISOPA.xlsx
@@ -827,7 +827,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Nueva base: PROCEDIMIENTO I.pdf, 14 páginas. Las siete plantillas anteriores se retiraron del catálogo activo. El llenado aún está pendiente de adaptar.</t>
+          <t>Base activa: PROCEDIMIENTO I.pdf, 14 páginas. El formulario genera PDF directamente; las siete plantillas Word anteriores se retiraron.</t>
         </is>
       </c>
     </row>
@@ -4659,7 +4659,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nueva base PDF; llenado pendiente de configurar</t>
+          <t>PDF nativo: usar formulario; 14 páginas; hasta 5 asistentes</t>
         </is>
       </c>
     </row>
@@ -4731,8 +4731,6 @@
           <t>POL-I</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Politica</t>

</xml_diff>

<commit_message>
Integrate SASISOPA1 PDF batch with selection and merged output
</commit_message>
<xml_diff>
--- a/Base_SASISOPA.xlsx
+++ b/Base_SASISOPA.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Completa las hojas con datos reales. Este archivo es la base; todavía no genera documentos Word.</t>
+          <t>Base actual: tres PDF de SASISOPA1, 87 páginas. Captura en Iniciar.bat; Excel se conserva como catálogo, sin importación de datos en este modo.</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4630,36 +4630,70 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>plantilla_id</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>archivo_word</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>hojas_datos</t>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>archivo_pdf</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>uso</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>POL-I</t>
+          <t>POL-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PROCEDIMIENTO I.pdf</t>
+          <t>1 POLITICA.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PDF nativo: usar formulario; 14 páginas; hasta 5 asistentes</t>
+          <t>Formulario PDF: 14 páginas; campos vacíos conservan el original</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PEL-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2. ID DE PELIGROS.pdf</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Formulario PDF: 53 páginas; campos vacíos conservan el original</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LEG-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3. REQUISITOS LEGALES.pdf</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Formulario PDF: 20 páginas; campos vacíos conservan el original</t>
         </is>
       </c>
     </row>
@@ -4677,7 +4711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4728,15 +4762,59 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>POL-I</t>
+          <t>POL-01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Politica</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SOL-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PEL-02</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Identificación de peligros</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SOL-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LEG-03</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Requisitos legales</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Integrate 18 SASISOPA PDFs with role-based editor and ZIP import
</commit_message>
<xml_diff>
--- a/Base_SASISOPA.xlsx
+++ b/Base_SASISOPA.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Base actual: tres PDF de SASISOPA1, 87 páginas. Captura en Iniciar.bat; Excel se conserva como catálogo, sin importación de datos en este modo.</t>
+          <t>Base activa: 18 PDF limpios, 523 páginas. Importar SASISOPA.zip desde Iniciar.bat; capturar por estación, personas y funciones. Excel es catálogo, sin importación automática.</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4649,51 +4649,306 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>POL-01</t>
+          <t>I</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1 POLITICA.pdf</t>
+          <t>PROCEDIMIENTO I.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Formulario PDF: 14 páginas; campos vacíos conservan el original</t>
+          <t>Base limpia: 14 páginas; usar editor de datos y funciones</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PEL-02</t>
+          <t>II</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2. ID DE PELIGROS.pdf</t>
+          <t>PROCEDIMIENTO II.pdf</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Formulario PDF: 53 páginas; campos vacíos conservan el original</t>
+          <t>Base limpia: 57 páginas; usar editor de datos y funciones</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LEG-03</t>
+          <t>III</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3. REQUISITOS LEGALES.pdf</t>
+          <t>PROCEDIMIENTO III.pdf</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Formulario PDF: 20 páginas; campos vacíos conservan el original</t>
+          <t>Base limpia: 26 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO IV.pdf</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Base limpia: 13 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO V.pdf</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Base limpia: 21 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO VI.pdf</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Base limpia: 45 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>VII</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO VII.pdf</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Base limpia: 15 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VIII</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO VIII.pdf</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Base limpia: 18 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>IX</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO IX.pdf</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Base limpia: 16 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO X.pdf</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Base limpia: 24 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>XI</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO XI.pdf</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Base limpia: 33 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>XII</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO XII.pdf</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Base limpia: 44 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>XIII</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO XIII.pdf</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Base limpia: 70 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>XIV</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO XIV.pdf</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Base limpia: 39 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>XV</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO XV.pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Base limpia: 31 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>XVI</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO XVI.pdf</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Base limpia: 39 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>XVII</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO XVII.pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Base limpia: 10 páginas; usar editor de datos y funciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>XVIII</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PROCEDIMIENTO XVIII.pdf</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Base limpia: 8 páginas; usar editor de datos y funciones</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4762,7 +5017,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>POL-01</t>
+          <t>I</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -4784,12 +5039,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PEL-02</t>
+          <t>II</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Identificación de peligros</t>
+          <t>Peligros y riesgos</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4806,7 +5061,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LEG-03</t>
+          <t>III</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -4815,6 +5070,336 @@
         </is>
       </c>
       <c r="F4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SOL-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Objetivos, metas e indicadores</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SOL-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Funciones y autoridad</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SOL-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Competencia y capacitación</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SOL-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>VII</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Comunicación</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SOL-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>VIII</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Control documental</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SOL-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>IX</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Mejores prácticas</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SOL-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Control de actividades y procesos</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SOL-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>XI</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Integridad mecánica</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SOL-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>XII</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Contratistas</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SOL-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>XIII</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Emergencias</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SOL-014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>XIV</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Monitoreo y evaluación</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SOL-015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>XV</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Auditorías</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SOL-016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>XVI</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Incidentes y accidentes</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SOL-017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>XVII</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Revisión de resultados</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SOL-018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>XVIII</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Informe de desempeño</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>